<commit_message>
Bump nav.js to v=3 to refresh cached active-section highlight
Force browsers to refetch nav.js so the current-section highlight
(amber, bold) actually shows. No underline.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Employees/Employee_View.xlsx
+++ b/Employees/Employee_View.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\.My computer\Vulyk Clinic Website\Employees\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{711100E9-6CC8-4657-A02F-D646E79DDA3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F3E8029-D62B-4A9C-988F-6AB89980163C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="386">
   <si>
     <t>Employee View</t>
   </si>
@@ -1150,9 +1150,6 @@
     <t>Дорослий та дитячий хірург</t>
   </si>
   <si>
-    <t>Медсестра (в декруті)</t>
-  </si>
-  <si>
     <t>Менеджер з адміністративної діяльності</t>
   </si>
   <si>
@@ -1171,10 +1168,16 @@
     <t>Тавридзька</t>
   </si>
   <si>
-    <t>Дитячий психотерапевт</t>
-  </si>
-  <si>
     <t>Медична Директор, Сімейна лікарка</t>
+  </si>
+  <si>
+    <t>Дитячий психіатр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Медсестра </t>
+  </si>
+  <si>
+    <t>Тичини (декрет)</t>
   </si>
 </sst>
 </file>
@@ -1568,7 +1571,7 @@
   <cols>
     <col min="4" max="4" width="13.5546875" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" customWidth="1"/>
+    <col min="9" max="9" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" x14ac:dyDescent="0.3">
@@ -2313,10 +2316,10 @@
         <v>50</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>367</v>
+        <v>385</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>52</v>
@@ -2396,7 +2399,7 @@
         <v>62</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>367</v>
@@ -2668,7 +2671,7 @@
         <v>144</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="I18" t="s">
         <v>372</v>
@@ -3505,7 +3508,7 @@
         <v>62</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>368</v>
@@ -3771,7 +3774,7 @@
         <v>110</v>
       </c>
       <c r="I34" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="J34" s="3" t="s">
         <v>52</v>
@@ -4461,7 +4464,7 @@
         <v>62</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="I46" s="3" t="s">
         <v>367</v>
@@ -4540,13 +4543,13 @@
         <v>96</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>81</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="I48" s="3" t="s">
         <v>368</v>
@@ -4557,7 +4560,7 @@
         <v>123</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>81</v>

</xml_diff>